<commit_message>
Deleted correlations to Wyangala and flood correlations between Hay and Redbank as in both of these situations, data gaps prevent Wyangala/Hay from extending the dataset so correlations are pointless
</commit_message>
<xml_diff>
--- a/raw/trend_analysis.xlsx
+++ b/raw/trend_analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/cumbung_assessment/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="240" documentId="8_{4CC3F85E-C413-4D2C-B6D6-BE92EA178B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01C5021C-C732-4368-AA41-DF229CD29E7D}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="8_{4CC3F85E-C413-4D2C-B6D6-BE92EA178B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDB912AB-117A-423C-B533-DF6223E7C5E3}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="8" xr2:uid="{DAE106E8-A078-4344-BC5B-36A76772C6D7}"/>
+    <workbookView xWindow="768" yWindow="444" windowWidth="19740" windowHeight="13356" firstSheet="1" activeTab="8" xr2:uid="{DAE106E8-A078-4344-BC5B-36A76772C6D7}"/>
   </bookViews>
   <sheets>
     <sheet name="cumbung" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="11">
   <si>
     <t>Year</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>Inun_area</t>
-  </si>
-  <si>
-    <t>year</t>
   </si>
   <si>
     <t>Flood</t>
@@ -5566,7 +5563,7 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -6182,16 +6179,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
         <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -7486,10 +7483,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -8054,7 +8051,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -8933,7 +8930,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -9783,16 +9780,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
         <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -10672,7 +10669,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -11188,7 +11185,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -12470,16 +12467,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
-        <v>10</v>
-      </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>